<commit_message>
Sizes read Width then Length everywhere operators look
Operators read sizes as W x L. Display and entry order only; stored L/W unchanged,
so cutting, edge banding and pricing do not move.

- Cutting List entry grid, block paste order, HPL builds table: Width before Length
- Excel template (file + fallback) and HPL sheet: Width column before Length.
  Panel upload already reads by header; HPL upload now reads the header so old
  Length-first files still import the right way round
- Job Order parts table, Excel/CSV export, part labels (text + QR size), board
  diagram piece labels, cut-sheet parts list, analysis review table + export,
  client-list import preview, Read drawing check window, fit warning
- smoke: board label now 400x600; new check for paste order/template/JO header

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cutting-List-Template.xlsx
+++ b/Cutting-List-Template.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Width (mm)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Length (mm)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Width (mm)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -552,10 +552,10 @@
         <v>2</v>
       </c>
       <c r="F2" t="n">
+        <v>560</v>
+      </c>
+      <c r="G2" t="n">
         <v>720</v>
-      </c>
-      <c r="G2" t="n">
-        <v>560</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -606,10 +606,10 @@
         <v>2</v>
       </c>
       <c r="F3" t="n">
+        <v>296</v>
+      </c>
+      <c r="G3" t="n">
         <v>716</v>
-      </c>
-      <c r="G3" t="n">
-        <v>296</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -679,12 +679,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Width (mm)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Length (mm)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Width (mm)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -847,7 +847,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -876,7 +875,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>